<commit_message>
feat(central): update budget actuals logic, UI enhancements, NDT filters and memo history
</commit_message>
<xml_diff>
--- a/home/src/site_apps/central/data/Material_Inventory.xlsx
+++ b/home/src/site_apps/central/data/Material_Inventory.xlsx
@@ -27309,25 +27309,25 @@
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>9441641</v>
+        <v>13575105</v>
       </c>
       <c r="N2" t="n">
-        <v>9441641</v>
+        <v>13575105</v>
       </c>
       <c r="O2" t="n">
-        <v>2615334</v>
+        <v>3268210</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>707019</v>
+        <v>1722002</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>6119288</v>
+        <v>0</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
@@ -27338,7 +27338,7 @@
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
-          <t>{"\uc774\uc0ac": {"personnel": "", "period": "", "unit_price": 230208.33333333334}, "\ubd80\uc7a5": {"personnel": "2", "period": "4.5", "unit_price": 230208.33333333334}, "\ucc28\uc7a5": {"personnel": "", "period": "", "unit_price": 198625.0}, "\uacfc\uc7a5": {"personnel": "", "period": "", "unit_price": 171541.66666666666}, "\ub300\ub9ac": {"personnel": "", "period": "", "unit_price": 158000.0}, "\uacc4\uc7a5": {"personnel": "1", "period": "1", "unit_price": 144458.33333333334}, "\uc8fc\uc784": {"personnel": "", "period": "", "unit_price": 130916.66666666667}, "\uae30\uc0ac": {"personnel": "", "period": "", "unit_price": 121875.0}, "\uc5f0\uc7a5\uadfc\ubb34": {"personnel": "2", "period": "3", "unit_price": 4000.0}, "\uc57c\uac04\uadfc\ubb34": {"personnel": "", "period": "", "unit_price": 5000.0}, "\ud734\uc77c\uadfc\ubb34": {"personnel": "3", "period": "16.6667", "unit_price": 7500.0}}</t>
+          <t>{"\uc774\uc0ac": {"personnel": "", "period": "", "unit_price": 230208.33333333334}, "\ubd80\uc7a5": {"personnel": "2", "period": "5.5", "unit_price": 230208.33333333334}, "\ucc28\uc7a5": {"personnel": "", "period": "", "unit_price": 198625.0}, "\uacfc\uc7a5": {"personnel": "", "period": "", "unit_price": 171541.66666666666}, "\ub300\ub9ac": {"personnel": "", "period": "", "unit_price": 158000.0}, "\uacc4\uc7a5": {"personnel": "1", "period": "2", "unit_price": 144458.33333333334}, "\uc8fc\uc784": {"personnel": "", "period": "", "unit_price": 130916.66666666667}, "\uae30\uc0ac": {"personnel": "", "period": "", "unit_price": 121875.0}, "\uc5f0\uc7a5\uadfc\ubb34": {"personnel": "3", "period": "6", "unit_price": 4000.0}, "\uc57c\uac04\uadfc\ubb34": {"personnel": "", "period": "", "unit_price": 5000.0}, "\ud734\uc77c\uadfc\ubb34": {"personnel": "3", "period": "16.6667", "unit_price": 7500.0}}</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -27348,7 +27348,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>{"site_expense": [{"cat": "\ucc28\ub7c9\uc720\uc9c0\ube44", "cont": "\uc8fc\uc720, \uc218\ub9ac, \ud1b5\ud589, \uc8fc\ucc28 \ub4f1", "ppl": "N/A", "qty": "6", "unit": "\uc77c", "price": "6667", "amount": "40,002"}, {"cat": "\uc18c\ubaa8\ud488\ube44", "cont": "\uc7a5\uac11,\uc77c\ud68c\uc6a9 \uc791\uc5c5\ubcf5\uc678", "ppl": "N/A", "qty": "6", "unit": "\uc77c", "price": "3333", "amount": "19,998"}, {"cat": "\ubcf5\ub9ac\ud6c4\uc0dd\ube44", "cont": "\uc0dd\uc218, \uc74c\ub8cc \uc678 \uae30\ud0c0", "ppl": "N/A", "qty": "6", "unit": "\uc77c", "price": "1667", "amount": "10,002"}, {"cat": "Se-175", "cont": "\ubc29\uc0ac\uc131\ub3d9\uc704\uc6d0\uc18c \uad6c\ub9e4", "ppl": "N/A", "qty": "", "unit": "\uc77c", "price": "35,714", "amount": "0"}], "rental": [{"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}], "outsource": [{"cat": "\ucf00\uc774\uc5d4\ub514\uc774", "work": "\ubc29\uc0ac\uc120\ud22c\uacfc\uac80\uc0ac", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}], "depreciation": [{"item": "PAUT \uc7a5\ube44", "spec": "", "life": "5", "qty": "1", "days": "5", "rate": "44,444", "amount": "222,222"}, {"item": "PAUT SCANNER (MANUAL)", "spec": "", "life": "5", "qty": "1", "days": "5", "rate": "5,556", "amount": "27,778"}, {"item": "PAUT SCANNER (COBRA)", "spec": "", "life": "5", "qty": "1", "days": "", "rate": "16,667", "amount": "0"}, {"item": "YOKE", "spec": "", "life": "5", "qty": "1", "days": "", "rate": "222", "amount": "0"}, {"item": "\ud604\uc0c1\uc6a9 \ud0d1\ucc28(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \ud0d1\ucc28 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "", "rate": "16,667", "amount": "0"}, {"item": "\uc2a4\ud0c0\ub809\uc2a4(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \uc2a4\ud0c0\ub809\uc2a4 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "6", "rate": "16,667", "amount": "100,000"}], "_depreciation_precise_rates": [44444.441666666666, 5555.558333333333, 16666.666666666668, 222.2, 16666.666666666668, 16666.66875]}</t>
+          <t>{"site_expense": [{"cat": "\ucc28\ub7c9\uc720\uc9c0\ube44", "cont": "\uc8fc\uc720, \uc218\ub9ac, \ud1b5\ud589, \uc8fc\ucc28 \ub4f1", "ppl": "4", "qty": "7", "unit": "\uc77c", "price": "6667", "amount": "46,669"}, {"cat": "\uc18c\ubaa8\ud488\ube44", "cont": "\uc7a5\uac11,\uc77c\ud68c\uc6a9 \uc791\uc5c5\ubcf5\uc678", "ppl": "N/A", "qty": "6", "unit": "\uac1c\uc6d4", "price": "100,000", "amount": "600,000"}, {"cat": "\ubcf5\ub9ac\ud6c4\uc0dd\ube44", "cont": "\uc0dd\uc218, \uc74c\ub8cc \uc678 \uae30\ud0c0", "ppl": "N/A", "qty": "6", "unit": "\uac1c\uc6d4", "price": "50,000", "amount": "300,000"}, {"cat": "Se-175", "cont": "\ubc29\uc0ac\uc131\ub3d9\uc704\uc6d0\uc18c \uad6c\ub9e4", "ppl": "N/A", "qty": "", "unit": "\uc77c", "price": "35,714", "amount": "0"}], "rental": [{"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}], "outsource": [{"cat": "\ucf00\uc774\uc5d4\ub514\uc774", "work": "\ubc29\uc0ac\uc120\ud22c\uacfc\uac80\uc0ac", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}], "depreciation": [{"item": "PAUT \uc7a5\ube44", "spec": "", "life": "5", "qty": "1", "days": "6", "rate": "44,444", "amount": "266,667"}, {"item": "PAUT SCANNER (MANUAL)", "spec": "", "life": "5", "qty": "1", "days": "6", "rate": "5,556", "amount": "33,333"}, {"item": "PAUT SCANNER (COBRA)", "spec": "", "life": "5", "qty": "1", "days": "", "rate": "16,667", "amount": "0"}, {"item": "YOKE", "spec": "", "life": "5", "qty": "1", "days": "", "rate": "222", "amount": "0"}, {"item": "\ud604\uc0c1\uc6a9 \ud0d1\ucc28(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \ud0d1\ucc28 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "", "rate": "16,667", "amount": "0"}, {"item": "\uc2a4\ud0c0\ub809\uc2a4(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \uc2a4\ud0c0\ub809\uc2a4 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "7", "rate": "16,667", "amount": "116,667"}], "_depreciation_precise_rates": [44444.441666666666, 5555.558333333333, 16666.666666666668, 222.2, 16666.666666666668, 16666.66875]}</t>
         </is>
       </c>
     </row>
@@ -27396,10 +27396,10 @@
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>13461323</v>
+        <v>13575105</v>
       </c>
       <c r="N3" t="n">
-        <v>13461323</v>
+        <v>13575105</v>
       </c>
       <c r="O3" t="n">
         <v>3268210</v>

</xml_diff>

<commit_message>
Fix NDT billing export and GUI summary to group by inspection method and unit
</commit_message>
<xml_diff>
--- a/home/src/site_apps/central/data/Material_Inventory.xlsx
+++ b/home/src/site_apps/central/data/Material_Inventory.xlsx
@@ -24841,7 +24841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DE12"/>
+  <dimension ref="A1:DE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28268,6 +28268,273 @@
         <v>0</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>중앙지사</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>480</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.1546</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" s="1" t="n">
+        <v>46301.46898743055</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>PAUT MX2(OMNI2-103085)</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>2.1546</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>270981</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" t="n">
+        <v>583855</v>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>PAUT</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>(휴일) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>67,500</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>부장 이병국</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>(휴일) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>67,500</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="inlineStr"/>
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr"/>
+      <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr"/>
+      <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
+      <c r="AZ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG13" t="inlineStr">
+        <is>
+          <t>90서8616 (스타렉스) || 개인차량(이병국부장)</t>
+        </is>
+      </c>
+      <c r="BH13" t="inlineStr">
+        <is>
+          <t>60 ||</t>
+        </is>
+      </c>
+      <c r="BI13" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함 || out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호</t>
+        </is>
+      </c>
+      <c r="BJ13" t="inlineStr">
+        <is>
+          <t>||</t>
+        </is>
+      </c>
+      <c r="BK13" t="inlineStr"/>
+      <c r="BL13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM13" t="inlineStr"/>
+      <c r="BN13" t="inlineStr">
+        <is>
+          <t>한국지역난방공사 중앙지사</t>
+        </is>
+      </c>
+      <c r="BO13" t="inlineStr"/>
+      <c r="BP13" t="inlineStr"/>
+      <c r="BQ13" t="inlineStr"/>
+      <c r="BR13" t="inlineStr"/>
+      <c r="BS13" t="inlineStr"/>
+      <c r="BT13" t="inlineStr"/>
+      <c r="BU13" t="inlineStr"/>
+      <c r="BV13" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="BW13" t="inlineStr">
+        <is>
+          <t>KS B ISO 13588</t>
+        </is>
+      </c>
+      <c r="BX13" t="inlineStr"/>
+      <c r="BY13" t="inlineStr"/>
+      <c r="BZ13" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="CA13" t="inlineStr"/>
+      <c r="CB13" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC13" t="inlineStr">
+        <is>
+          <t>100A 이하 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD13" t="inlineStr"/>
+      <c r="CE13" t="inlineStr"/>
+      <c r="CF13" t="inlineStr"/>
+      <c r="CG13" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH13" t="n">
+        <v>2.1546</v>
+      </c>
+      <c r="CI13" t="n">
+        <v>82368</v>
+      </c>
+      <c r="CJ13" t="n">
+        <v>199003</v>
+      </c>
+      <c r="CK13" t="n">
+        <v>218903</v>
+      </c>
+      <c r="CL13" t="n">
+        <v>83581</v>
+      </c>
+      <c r="CM13" t="inlineStr"/>
+      <c r="CN13" t="inlineStr"/>
+      <c r="CO13" t="inlineStr"/>
+      <c r="CP13" t="inlineStr"/>
+      <c r="CQ13" t="inlineStr"/>
+      <c r="CR13" t="inlineStr"/>
+      <c r="CS13" t="inlineStr"/>
+      <c r="CT13" t="inlineStr"/>
+      <c r="CU13" t="inlineStr"/>
+      <c r="CV13" t="inlineStr"/>
+      <c r="CW13" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX13" t="n">
+        <v>6</v>
+      </c>
+      <c r="CY13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ13" t="inlineStr">
+        <is>
+          <t>100A</t>
+        </is>
+      </c>
+      <c r="DA13" t="inlineStr">
+        <is>
+          <t>열배관</t>
+        </is>
+      </c>
+      <c r="DB13" t="inlineStr"/>
+      <c r="DC13" t="inlineStr"/>
+      <c r="DD13" t="inlineStr"/>
+      <c r="DE13" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>